<commit_message>
06 Phase 5 Completed Data Format Standardization
</commit_message>
<xml_diff>
--- a/data/processed/cleaned_dataset.xlsx
+++ b/data/processed/cleaned_dataset.xlsx
@@ -2981,7 +2981,7 @@
         </is>
       </c>
       <c r="N41" t="n">
-        <v>769.3799999999999</v>
+        <v>769.38</v>
       </c>
     </row>
     <row r="42">
@@ -4655,7 +4655,7 @@
         </is>
       </c>
       <c r="N68" t="n">
-        <v>635.9000000000001</v>
+        <v>635.9</v>
       </c>
     </row>
     <row r="69">
@@ -5833,7 +5833,7 @@
         </is>
       </c>
       <c r="N87" t="n">
-        <v>440.1899999999999</v>
+        <v>440.19</v>
       </c>
     </row>
     <row r="88">
@@ -7445,7 +7445,7 @@
         </is>
       </c>
       <c r="N113" t="n">
-        <v>927.6600000000001</v>
+        <v>927.66</v>
       </c>
     </row>
     <row r="114">
@@ -7569,7 +7569,7 @@
         </is>
       </c>
       <c r="N115" t="n">
-        <v>950.4000000000001</v>
+        <v>950.4</v>
       </c>
     </row>
     <row r="116">
@@ -8189,7 +8189,7 @@
         </is>
       </c>
       <c r="N125" t="n">
-        <v>834.1200000000001</v>
+        <v>834.12</v>
       </c>
     </row>
     <row r="126">
@@ -12343,7 +12343,7 @@
         </is>
       </c>
       <c r="N192" t="n">
-        <v>671.0999999999999</v>
+        <v>671.1</v>
       </c>
     </row>
     <row r="193">
@@ -13087,7 +13087,7 @@
         </is>
       </c>
       <c r="N204" t="n">
-        <v>761.9399999999999</v>
+        <v>761.9400000000001</v>
       </c>
     </row>
     <row r="205">
@@ -14513,7 +14513,7 @@
         </is>
       </c>
       <c r="N227" t="n">
-        <v>821.8799999999999</v>
+        <v>821.88</v>
       </c>
     </row>
     <row r="228">
@@ -16311,7 +16311,7 @@
         </is>
       </c>
       <c r="N256" t="n">
-        <v>789.5699999999999</v>
+        <v>789.5700000000001</v>
       </c>
     </row>
     <row r="257">
@@ -19783,7 +19783,7 @@
         </is>
       </c>
       <c r="N312" t="n">
-        <v>397.4399999999999</v>
+        <v>397.44</v>
       </c>
     </row>
     <row r="313">
@@ -22387,7 +22387,7 @@
         </is>
       </c>
       <c r="N354" t="n">
-        <v>869.8000000000001</v>
+        <v>869.8</v>
       </c>
     </row>
     <row r="355">
@@ -28401,7 +28401,7 @@
         </is>
       </c>
       <c r="N451" t="n">
-        <v>759.1500000000001</v>
+        <v>759.15</v>
       </c>
     </row>
     <row r="452">
@@ -32431,7 +32431,7 @@
         </is>
       </c>
       <c r="N516" t="n">
-        <v>912.4499999999999</v>
+        <v>912.45</v>
       </c>
     </row>
     <row r="517">
@@ -37267,7 +37267,7 @@
         </is>
       </c>
       <c r="N594" t="n">
-        <v>612.8100000000001</v>
+        <v>612.8099999999999</v>
       </c>
     </row>
     <row r="595">
@@ -38011,7 +38011,7 @@
         </is>
       </c>
       <c r="N606" t="n">
-        <v>97.85999999999999</v>
+        <v>97.86</v>
       </c>
     </row>
     <row r="607">
@@ -54565,7 +54565,7 @@
         </is>
       </c>
       <c r="N873" t="n">
-        <v>972.9000000000001</v>
+        <v>972.9</v>
       </c>
     </row>
     <row r="874">
@@ -54813,7 +54813,7 @@
         </is>
       </c>
       <c r="N877" t="n">
-        <v>666.9499999999999</v>
+        <v>666.95</v>
       </c>
     </row>
     <row r="878">
@@ -58719,7 +58719,7 @@
         </is>
       </c>
       <c r="N940" t="n">
-        <v>994.3799999999999</v>
+        <v>994.38</v>
       </c>
     </row>
     <row r="941">
@@ -62005,7 +62005,7 @@
         </is>
       </c>
       <c r="N993" t="n">
-        <v>635.9000000000001</v>
+        <v>635.9</v>
       </c>
     </row>
     <row r="994">
@@ -62129,7 +62129,7 @@
         </is>
       </c>
       <c r="N995" t="n">
-        <v>802.3499999999999</v>
+        <v>802.35</v>
       </c>
     </row>
     <row r="996">
@@ -63679,7 +63679,7 @@
         </is>
       </c>
       <c r="N1020" t="n">
-        <v>547.4399999999999</v>
+        <v>547.4400000000001</v>
       </c>
     </row>
     <row r="1021">
@@ -68205,7 +68205,7 @@
         </is>
       </c>
       <c r="N1093" t="n">
-        <v>628.4399999999999</v>
+        <v>628.4400000000001</v>
       </c>
     </row>
     <row r="1094">
@@ -69879,7 +69879,7 @@
         </is>
       </c>
       <c r="N1120" t="n">
-        <v>754.4399999999999</v>
+        <v>754.4400000000001</v>
       </c>
     </row>
     <row r="1121">
@@ -70375,7 +70375,7 @@
         </is>
       </c>
       <c r="N1128" t="n">
-        <v>950.5500000000001</v>
+        <v>950.55</v>
       </c>
     </row>
     <row r="1129">
@@ -72297,7 +72297,7 @@
         </is>
       </c>
       <c r="N1159" t="n">
-        <v>904.6500000000001</v>
+        <v>904.65</v>
       </c>
     </row>
     <row r="1160">
@@ -72669,7 +72669,7 @@
         </is>
       </c>
       <c r="N1165" t="n">
-        <v>918.8700000000001</v>
+        <v>918.87</v>
       </c>
     </row>
     <row r="1166">
@@ -72855,7 +72855,7 @@
         </is>
       </c>
       <c r="N1168" t="n">
-        <v>973.4100000000001</v>
+        <v>973.41</v>
       </c>
     </row>
     <row r="1169">
@@ -74591,7 +74591,7 @@
         </is>
       </c>
       <c r="N1196" t="n">
-        <v>568.3199999999999</v>
+        <v>568.3200000000001</v>
       </c>
     </row>
     <row r="1197">

</xml_diff>